<commit_message>
modify the obj functions for max_st and min_em and add old growth yield'
</commit_message>
<xml_diff>
--- a/results/emission.xlsx
+++ b/results/emission.xlsx
@@ -474,10 +474,10 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>-2515007.418206576</v>
+        <v>-2019714.816200706</v>
       </c>
       <c r="F2" t="n">
-        <v>-2515007.418206576</v>
+        <v>-2019714.816200706</v>
       </c>
     </row>
     <row r="3">
@@ -485,19 +485,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>876663.5182445209</v>
+        <v>791652.6680417507</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>876663.5182445209</v>
+        <v>791652.6680417507</v>
       </c>
       <c r="E3" t="n">
-        <v>1306319.689602927</v>
+        <v>1188120.460265303</v>
       </c>
       <c r="F3" t="n">
-        <v>2182983.207847448</v>
+        <v>1979773.128307053</v>
       </c>
     </row>
     <row r="4">
@@ -505,19 +505,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>1165700.198931394</v>
+        <v>1054567.468695136</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>1165700.198931394</v>
+        <v>1054567.468695136</v>
       </c>
       <c r="E4" t="n">
-        <v>-401483.2380664512</v>
+        <v>-702868.5149176369</v>
       </c>
       <c r="F4" t="n">
-        <v>764216.9608649432</v>
+        <v>351698.9537774987</v>
       </c>
     </row>
     <row r="5">
@@ -525,19 +525,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>1390816.352275759</v>
+        <v>1272832.831514438</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>1390816.352275759</v>
+        <v>1272832.831514438</v>
       </c>
       <c r="E5" t="n">
-        <v>-1502979.778848212</v>
+        <v>-2174179.524067189</v>
       </c>
       <c r="F5" t="n">
-        <v>-112163.426572453</v>
+        <v>-901346.6925527507</v>
       </c>
     </row>
     <row r="6">
@@ -545,19 +545,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>1453091.396268783</v>
+        <v>1382552.921213425</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>1453091.396268783</v>
+        <v>1382552.921213425</v>
       </c>
       <c r="E6" t="n">
-        <v>-1473402.664590993</v>
+        <v>-1871728.971553548</v>
       </c>
       <c r="F6" t="n">
-        <v>-20311.26832220983</v>
+        <v>-489176.0503401237</v>
       </c>
     </row>
     <row r="7">
@@ -565,19 +565,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>1485408.60282823</v>
+        <v>1452706.838984197</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>1485408.60282823</v>
+        <v>1452706.838984197</v>
       </c>
       <c r="E7" t="n">
-        <v>-759328.4909590487</v>
+        <v>-1207807.030302483</v>
       </c>
       <c r="F7" t="n">
-        <v>726080.1118691813</v>
+        <v>244899.8086817143</v>
       </c>
     </row>
     <row r="8">
@@ -585,19 +585,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>1417358.485838958</v>
+        <v>1451823.697888546</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>1417358.485838958</v>
+        <v>1451823.697888546</v>
       </c>
       <c r="E8" t="n">
-        <v>-2833412.93896434</v>
+        <v>-2206012.985446376</v>
       </c>
       <c r="F8" t="n">
-        <v>-1416054.453125382</v>
+        <v>-754189.2875578299</v>
       </c>
     </row>
     <row r="9">
@@ -605,19 +605,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>1486404.488605577</v>
+        <v>1452650.378585598</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>1486404.488605577</v>
+        <v>1452650.378585598</v>
       </c>
       <c r="E9" t="n">
-        <v>-1444270.181108203</v>
+        <v>-3522429.090046758</v>
       </c>
       <c r="F9" t="n">
-        <v>42134.30749737332</v>
+        <v>-2069778.71146116</v>
       </c>
     </row>
     <row r="10">
@@ -625,19 +625,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>1237228.929894109</v>
+        <v>1509225.476493221</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>1237228.929894109</v>
+        <v>1509225.476493221</v>
       </c>
       <c r="E10" t="n">
-        <v>-3076644.03439256</v>
+        <v>-2089942.958138658</v>
       </c>
       <c r="F10" t="n">
-        <v>-1839415.10449845</v>
+        <v>-580717.481645437</v>
       </c>
     </row>
     <row r="11">
@@ -645,19 +645,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>979493.4069906169</v>
+        <v>1256398.041396933</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>979493.4069906169</v>
+        <v>1256398.041396933</v>
       </c>
       <c r="E11" t="n">
-        <v>-7738433.732811249</v>
+        <v>-8209468.654733166</v>
       </c>
       <c r="F11" t="n">
-        <v>-6758940.325820632</v>
+        <v>-6953070.613336232</v>
       </c>
     </row>
   </sheetData>

</xml_diff>